<commit_message>
feat: atualizar visitantes e membros após 02/08/2026
Inclui 32 novos visitantes (04–09/08/2026) e 5 novas contagens de
participação por culto, regenerando KPIs e gráficos do dashboard.

Co-authored-by: Lucas Andrade Silva <LucasAndradeSilva@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/membros-2.0.xlsx
+++ b/membros-2.0.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -617,6 +617,161 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5838</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>04/08/2026 21:42</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>542</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Terça · Fé e Milagres</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>86</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5871</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>06/08/2026 21:44</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>282</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Quinta · Quinta Profética</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>34</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5905</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>08/08/2026 23:52</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>215</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sábado · Arena</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5906</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>09/08/2026 12:53</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>690</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Domingo · Culto da Família (Manhã)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>153</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5915</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>09/08/2026 23:25</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>223</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Culto da Família (Noite)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>42</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: atualizar visitantes e membros após 09/08/2026
Inclui 17 novos visitantes (11–16/08/2026) e 4 novas contagens de
participação por culto, regenerando KPIs e gráficos do dashboard.

Co-authored-by: Lucas Andrade Silva <LucasAndradeSilva@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/membros-2.0.xlsx
+++ b/membros-2.0.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -772,6 +772,130 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5993</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>11/08/2026 22:03</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>459</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Terça · Fé e Milagres</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>55</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>6054</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>13/08/2026 21:49</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>321</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Quinta · Quinta Profética</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>38</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6084</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16/08/2026 12:34</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>459</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Domingo · Culto da Família (Manhã)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>90</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>6088</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16/08/2026 20:35</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>212</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Culto da Família (Noite)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: atualizar visitantes e membros após 16/08/2026
Inclui 29 novos registros de visitantes (18–23/08/2026; 28 únicos após
dedupe) e 5 novas contagens de participação por culto, regenerando KPIs
e gráficos do dashboard.

Co-authored-by: Lucas Andrade Silva <LucasAndradeSilva@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/membros-2.0.xlsx
+++ b/membros-2.0.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -896,6 +896,161 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6146</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>18/08/2026 21:25</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>489</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Terça · Fé e Milagres</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>72</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>6204</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>21/08/2026 07:11</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>540</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Quinta · Quinta Profética</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>63</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6215</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>22/08/2026 21:06</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>168</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sábado · Arena</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>7</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>6236</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>23/08/2026 19:18</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>488</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Domingo · Culto da Família (Manhã)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>82</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>6243</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pessoa não cadastrada (CPF: Não informado)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23/08/2026 21:15</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>249</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Culto da Família (Noite)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>53</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>